<commit_message>
Update template and split quantity/unit into separate columns
New template adds separate 数量/单位 columns and a 总价 column.
Column mapping: D=数量 E=单位 F=单价 G=总价 H-O=金额拆位 P=备注.
Also updated to single-copy template layout.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/templates/送货单(三联针式打印)1.xlsx
+++ b/backend/templates/送货单(三联针式打印)1.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="27">
   <si>
     <t>武汉市长江新区宏远商贸商行</t>
   </si>
@@ -46,7 +46,7 @@
     <t xml:space="preserve">                    编号：</t>
   </si>
   <si>
-    <t>发往地址：                                             联系人：      电话：</t>
+    <t>发往地址：                                             联系人：             电话：</t>
   </si>
   <si>
     <t>序号</t>
@@ -55,13 +55,22 @@
     <t>商品名称/型号</t>
   </si>
   <si>
-    <t>数量/单位</t>
+    <t>数量</t>
+  </si>
+  <si>
+    <t>单位</t>
   </si>
   <si>
     <t>单价</t>
   </si>
   <si>
+    <t>总价</t>
+  </si>
+  <si>
     <t>金额</t>
+  </si>
+  <si>
+    <t>备注</t>
   </si>
   <si>
     <t>拾</t>
@@ -145,7 +154,7 @@
         <rFont val="微软雅黑"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">          第二联：客户 </t>
+      <t xml:space="preserve">            第二联：客户 </t>
     </r>
     <r>
       <rPr>
@@ -161,7 +170,7 @@
         <rFont val="微软雅黑"/>
         <charset val="134"/>
       </rPr>
-      <t xml:space="preserve">            第三联：财务</t>
+      <t xml:space="preserve">        第三联：财务</t>
     </r>
     <r>
       <rPr>
@@ -805,7 +814,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -830,14 +839,26 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1">
       <alignment vertical="center"/>
@@ -1207,23 +1228,25 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:M37"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.25"/>
+  <dimension ref="B2:P20"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="17.4"/>
   <cols>
     <col min="1" max="1" width="2.6" style="1" customWidth="1"/>
     <col min="2" max="2" width="11" style="1" customWidth="1"/>
     <col min="3" max="3" width="29.75" style="1" customWidth="1"/>
-    <col min="4" max="4" width="10.25" style="1" customWidth="1"/>
-    <col min="5" max="5" width="9.5" style="1" customWidth="1"/>
-    <col min="6" max="7" width="3.25" style="1" customWidth="1"/>
-    <col min="8" max="11" width="3" style="1" customWidth="1"/>
-    <col min="12" max="12" width="3.125" style="1" customWidth="1"/>
-    <col min="13" max="13" width="3.375" style="1" customWidth="1"/>
-    <col min="14" max="14" width="9.5" style="1" customWidth="1"/>
-    <col min="15" max="16384" width="9" style="1"/>
+    <col min="4" max="4" width="7.9" style="1" customWidth="1"/>
+    <col min="5" max="5" width="8.2" style="1" customWidth="1"/>
+    <col min="6" max="6" width="8" style="1" customWidth="1"/>
+    <col min="7" max="7" width="8.4" style="1" customWidth="1"/>
+    <col min="8" max="9" width="3.25" style="1" customWidth="1"/>
+    <col min="10" max="13" width="3" style="1" customWidth="1"/>
+    <col min="14" max="14" width="3.125" style="1" customWidth="1"/>
+    <col min="15" max="15" width="3.375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="9.5" style="1" customWidth="1"/>
+    <col min="17" max="16384" width="9" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" ht="24.75" spans="2:13">
+    <row r="2" ht="18.75" customHeight="1" spans="2:16">
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
@@ -1238,8 +1261,10 @@
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
       <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
     </row>
-    <row r="3" ht="31.5" customHeight="1" spans="2:13">
+    <row r="3" ht="31.5" customHeight="1" spans="2:16">
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
@@ -1254,8 +1279,10 @@
       <c r="K3" s="4"/>
       <c r="L3" s="4"/>
       <c r="M3" s="4"/>
+      <c r="N3" s="4"/>
+      <c r="O3" s="4"/>
     </row>
-    <row r="4" ht="14.25" customHeight="1" spans="2:13">
+    <row r="4" ht="14.25" customHeight="1" spans="2:16">
       <c r="B4" s="5" t="s">
         <v>2</v>
       </c>
@@ -1270,15 +1297,16 @@
       <c r="K4" s="5"/>
       <c r="L4" s="5"/>
       <c r="M4" s="5"/>
+      <c r="N4" s="5"/>
+      <c r="O4" s="5"/>
     </row>
-    <row r="5" ht="21.75" customHeight="1" spans="2:13">
+    <row r="5" ht="21.75" customHeight="1" spans="2:16">
       <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="6"/>
       <c r="F5" s="6"/>
       <c r="G5" s="6"/>
       <c r="H5" s="6"/>
@@ -1287,523 +1315,275 @@
       <c r="K5" s="6"/>
       <c r="L5" s="6"/>
       <c r="M5" s="6"/>
+      <c r="N5" s="6"/>
+      <c r="O5" s="6"/>
     </row>
-    <row r="6" ht="21" customHeight="1" spans="2:13">
+    <row r="6" ht="21" customHeight="1" spans="2:16">
       <c r="B6" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" customHeight="1" spans="2:13">
+    <row r="7" ht="17.25" customHeight="1" spans="2:16">
       <c r="B7" s="7" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="8" t="s">
         <v>8</v>
       </c>
       <c r="E7" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="8" t="s">
+      <c r="F7" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="G7" s="8"/>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="G7" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="I7" s="10"/>
+      <c r="J7" s="10"/>
+      <c r="K7" s="10"/>
+      <c r="L7" s="10"/>
+      <c r="M7" s="10"/>
+      <c r="N7" s="10"/>
+      <c r="O7" s="10"/>
+      <c r="P7" s="11" t="s">
+        <v>13</v>
+      </c>
     </row>
-    <row r="8" customHeight="1" spans="2:13">
-      <c r="B8" s="9"/>
-      <c r="C8" s="9"/>
-      <c r="D8" s="9"/>
-      <c r="E8" s="9"/>
-      <c r="F8" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="H8" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="I8" s="10" t="s">
+    <row r="8" ht="17.25" customHeight="1" spans="2:16">
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="12"/>
+      <c r="F8" s="12"/>
+      <c r="G8" s="14"/>
+      <c r="H8" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="J8" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="K8" s="10" t="s">
+      <c r="I8" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="L8" s="10" t="s">
+      <c r="J8" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="M8" s="10" t="s">
+      <c r="K8" s="11" t="s">
         <v>17</v>
       </c>
+      <c r="L8" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="M8" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="N8" s="11" t="s">
+        <v>19</v>
+      </c>
+      <c r="O8" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="P8" s="11"/>
     </row>
-    <row r="9" customHeight="1" spans="2:13">
-      <c r="B9" s="8">
+    <row r="9" ht="17.25" customHeight="1" spans="2:16">
+      <c r="B9" s="10">
         <v>1</v>
       </c>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10"/>
-      <c r="L9" s="10"/>
-      <c r="M9" s="10"/>
+      <c r="C9" s="11"/>
+      <c r="D9" s="11"/>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="11"/>
+      <c r="M9" s="11"/>
+      <c r="N9" s="11"/>
+      <c r="O9" s="11"/>
+      <c r="P9" s="11"/>
     </row>
-    <row r="10" customHeight="1" spans="2:13">
-      <c r="B10" s="8">
+    <row r="10" ht="17.25" customHeight="1" spans="2:16">
+      <c r="B10" s="10">
         <v>2</v>
       </c>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="10"/>
-      <c r="M10" s="10"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11"/>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11"/>
+      <c r="M10" s="11"/>
+      <c r="N10" s="11"/>
+      <c r="O10" s="11"/>
+      <c r="P10" s="11"/>
     </row>
-    <row r="11" ht="16.5" customHeight="1" spans="2:13">
-      <c r="B11" s="8">
+    <row r="11" ht="16.5" customHeight="1" spans="2:16">
+      <c r="B11" s="10">
         <v>3</v>
       </c>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="10"/>
-      <c r="M11" s="10"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11"/>
+      <c r="K11" s="11"/>
+      <c r="L11" s="11"/>
+      <c r="M11" s="11"/>
+      <c r="N11" s="11"/>
+      <c r="O11" s="11"/>
+      <c r="P11" s="11"/>
     </row>
-    <row r="12" customHeight="1" spans="2:13">
-      <c r="B12" s="8">
+    <row r="12" ht="17.25" customHeight="1" spans="2:16">
+      <c r="B12" s="10">
         <v>4</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10"/>
-      <c r="K12" s="10"/>
-      <c r="L12" s="10"/>
-      <c r="M12" s="10"/>
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+      <c r="L12" s="11"/>
+      <c r="M12" s="11"/>
+      <c r="N12" s="11"/>
+      <c r="O12" s="11"/>
+      <c r="P12" s="11"/>
     </row>
-    <row r="13" customHeight="1" spans="2:13">
-      <c r="B13" s="8">
+    <row r="13" ht="17.25" customHeight="1" spans="2:16">
+      <c r="B13" s="10">
         <v>5</v>
       </c>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10"/>
-      <c r="M13" s="10"/>
+      <c r="C13" s="11"/>
+      <c r="D13" s="11"/>
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="11"/>
+      <c r="M13" s="11"/>
+      <c r="N13" s="11"/>
+      <c r="O13" s="11"/>
+      <c r="P13" s="11"/>
     </row>
-    <row r="14" customHeight="1" spans="2:13">
-      <c r="B14" s="8">
+    <row r="14" ht="17.25" customHeight="1" spans="2:16">
+      <c r="B14" s="10">
         <v>6</v>
       </c>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="10"/>
-      <c r="L14" s="10"/>
-      <c r="M14" s="10"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="11"/>
+      <c r="M14" s="11"/>
+      <c r="N14" s="11"/>
+      <c r="O14" s="11"/>
+      <c r="P14" s="11"/>
     </row>
-    <row r="15" ht="23.25" customHeight="1" spans="2:13">
-      <c r="B15" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="10"/>
-      <c r="L15" s="10"/>
-      <c r="M15" s="10"/>
+    <row r="15" ht="23.25" customHeight="1" spans="2:16">
+      <c r="B15" s="10" t="s">
+        <v>21</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D15" s="11"/>
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="11"/>
+      <c r="M15" s="11"/>
+      <c r="N15" s="11"/>
+      <c r="O15" s="11"/>
+      <c r="P15" s="11"/>
     </row>
-    <row r="16" ht="18.75" customHeight="1" spans="2:13">
-      <c r="B16" s="11" t="s">
-        <v>20</v>
+    <row r="16" ht="18.75" customHeight="1" spans="2:16">
+      <c r="B16" s="15" t="s">
+        <v>23</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="E16" s="13"/>
-      <c r="F16" s="13"/>
-      <c r="G16" s="13"/>
-      <c r="H16" s="13"/>
-      <c r="I16" s="13"/>
-      <c r="J16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="13"/>
-      <c r="M16" s="13"/>
+        <v>24</v>
+      </c>
+      <c r="D16" s="4"/>
+      <c r="E16" s="16" t="s">
+        <v>25</v>
+      </c>
+      <c r="F16" s="17"/>
+      <c r="G16" s="17"/>
+      <c r="H16" s="17"/>
+      <c r="I16" s="17"/>
+      <c r="J16" s="17"/>
+      <c r="K16" s="17"/>
+      <c r="L16" s="17"/>
+      <c r="M16" s="17"/>
+      <c r="N16" s="17"/>
+      <c r="O16" s="17"/>
     </row>
-    <row r="17" ht="26.25" customHeight="1" spans="2:13">
-      <c r="B17" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
-      <c r="I17" s="14"/>
-      <c r="J17" s="14"/>
-      <c r="K17" s="14"/>
-      <c r="L17" s="14"/>
-      <c r="M17" s="14"/>
+    <row r="17" ht="26.25" customHeight="1" spans="2:15">
+      <c r="B17" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+      <c r="E17" s="18"/>
+      <c r="F17" s="18"/>
+      <c r="G17" s="18"/>
+      <c r="H17" s="18"/>
+      <c r="I17" s="18"/>
+      <c r="J17" s="18"/>
+      <c r="K17" s="18"/>
+      <c r="L17" s="18"/>
+      <c r="M17" s="18"/>
+      <c r="N17" s="18"/>
+      <c r="O17" s="18"/>
     </row>
     <row r="18" ht="20.1" customHeight="1"/>
     <row r="19" ht="20.1" customHeight="1"/>
     <row r="20" ht="20.1" customHeight="1"/>
-    <row r="21" ht="20.1" customHeight="1"/>
-    <row r="22" ht="18.75" customHeight="1" spans="2:13">
-      <c r="B22" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="2"/>
-      <c r="G22" s="2"/>
-      <c r="H22" s="2"/>
-      <c r="I22" s="2"/>
-      <c r="J22" s="2"/>
-      <c r="K22" s="2"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="2"/>
-    </row>
-    <row r="23" ht="31.5" customHeight="1" spans="2:13">
-      <c r="B23" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C23" s="4"/>
-      <c r="D23" s="4"/>
-      <c r="E23" s="4"/>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
-      <c r="M23" s="4"/>
-    </row>
-    <row r="24" ht="14.25" customHeight="1" spans="2:13">
-      <c r="B24" s="5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C24" s="5"/>
-      <c r="D24" s="5"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="5"/>
-      <c r="G24" s="5"/>
-      <c r="H24" s="5"/>
-      <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
-      <c r="K24" s="5"/>
-      <c r="L24" s="5"/>
-      <c r="M24" s="5"/>
-    </row>
-    <row r="25" ht="21.75" customHeight="1" spans="2:13">
-      <c r="B25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="E25" s="6"/>
-      <c r="F25" s="6"/>
-      <c r="G25" s="6"/>
-      <c r="H25" s="6"/>
-      <c r="I25" s="6"/>
-      <c r="J25" s="6"/>
-      <c r="K25" s="6"/>
-      <c r="L25" s="6"/>
-      <c r="M25" s="6"/>
-    </row>
-    <row r="26" ht="21" customHeight="1" spans="2:13">
-      <c r="B26" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" customHeight="1" spans="2:13">
-      <c r="B27" s="7" t="s">
-        <v>6</v>
-      </c>
-      <c r="C27" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="D27" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E27" s="7" t="s">
-        <v>9</v>
-      </c>
-      <c r="F27" s="8" t="s">
-        <v>10</v>
-      </c>
-      <c r="G27" s="8"/>
-      <c r="H27" s="8"/>
-      <c r="I27" s="8"/>
-      <c r="J27" s="8"/>
-      <c r="K27" s="8"/>
-      <c r="L27" s="8"/>
-      <c r="M27" s="8"/>
-    </row>
-    <row r="28" customHeight="1" spans="2:13">
-      <c r="B28" s="9"/>
-      <c r="C28" s="9"/>
-      <c r="D28" s="9"/>
-      <c r="E28" s="9"/>
-      <c r="F28" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G28" s="10" t="s">
-        <v>12</v>
-      </c>
-      <c r="H28" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="I28" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="J28" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="K28" s="10" t="s">
-        <v>15</v>
-      </c>
-      <c r="L28" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="M28" s="10" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="29" customHeight="1" spans="2:13">
-      <c r="B29" s="8">
-        <v>1</v>
-      </c>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10"/>
-      <c r="I29" s="10"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="10"/>
-      <c r="L29" s="10"/>
-      <c r="M29" s="10"/>
-    </row>
-    <row r="30" customHeight="1" spans="2:13">
-      <c r="B30" s="8">
-        <v>2</v>
-      </c>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="10"/>
-      <c r="H30" s="10"/>
-      <c r="I30" s="10"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="10"/>
-      <c r="L30" s="10"/>
-      <c r="M30" s="10"/>
-    </row>
-    <row r="31" ht="16.5" customHeight="1" spans="2:13">
-      <c r="B31" s="8">
-        <v>3</v>
-      </c>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="10"/>
-      <c r="H31" s="10"/>
-      <c r="I31" s="10"/>
-      <c r="J31" s="10"/>
-      <c r="K31" s="10"/>
-      <c r="L31" s="10"/>
-      <c r="M31" s="10"/>
-    </row>
-    <row r="32" customHeight="1" spans="2:13">
-      <c r="B32" s="8">
-        <v>4</v>
-      </c>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10"/>
-      <c r="H32" s="10"/>
-      <c r="I32" s="10"/>
-      <c r="J32" s="10"/>
-      <c r="K32" s="10"/>
-      <c r="L32" s="10"/>
-      <c r="M32" s="10"/>
-    </row>
-    <row r="33" customHeight="1" spans="2:13">
-      <c r="B33" s="8">
-        <v>5</v>
-      </c>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
-      <c r="H33" s="10"/>
-      <c r="I33" s="10"/>
-      <c r="J33" s="10"/>
-      <c r="K33" s="10"/>
-      <c r="L33" s="10"/>
-      <c r="M33" s="10"/>
-    </row>
-    <row r="34" customHeight="1" spans="2:13">
-      <c r="B34" s="8">
-        <v>6</v>
-      </c>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
-      <c r="F34" s="10"/>
-      <c r="G34" s="10"/>
-      <c r="H34" s="10"/>
-      <c r="I34" s="10"/>
-      <c r="J34" s="10"/>
-      <c r="K34" s="10"/>
-      <c r="L34" s="10"/>
-      <c r="M34" s="10"/>
-    </row>
-    <row r="35" ht="23.25" customHeight="1" spans="2:13">
-      <c r="B35" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="C35" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10"/>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
-      <c r="I35" s="10"/>
-      <c r="J35" s="10"/>
-      <c r="K35" s="10"/>
-      <c r="L35" s="10"/>
-      <c r="M35" s="10"/>
-    </row>
-    <row r="36" ht="18.75" customHeight="1" spans="2:13">
-      <c r="B36" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D36" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="E36" s="13"/>
-      <c r="F36" s="13"/>
-      <c r="G36" s="13"/>
-      <c r="H36" s="13"/>
-      <c r="I36" s="13"/>
-      <c r="J36" s="13"/>
-      <c r="K36" s="13"/>
-      <c r="L36" s="13"/>
-      <c r="M36" s="13"/>
-    </row>
-    <row r="37" ht="26.25" customHeight="1" spans="2:13">
-      <c r="B37" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="14"/>
-      <c r="J37" s="14"/>
-      <c r="K37" s="14"/>
-      <c r="L37" s="14"/>
-      <c r="M37" s="14"/>
-    </row>
   </sheetData>
-  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertRows="0" insertColumns="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
-  <mergeCells count="26">
-    <mergeCell ref="B2:M2"/>
-    <mergeCell ref="B3:M3"/>
-    <mergeCell ref="B4:M4"/>
-    <mergeCell ref="D5:M5"/>
-    <mergeCell ref="B6:M6"/>
-    <mergeCell ref="F7:M7"/>
-    <mergeCell ref="C15:E15"/>
-    <mergeCell ref="D16:M16"/>
-    <mergeCell ref="B17:M17"/>
-    <mergeCell ref="B22:M22"/>
-    <mergeCell ref="B23:M23"/>
-    <mergeCell ref="B24:M24"/>
-    <mergeCell ref="D25:M25"/>
-    <mergeCell ref="B26:M26"/>
-    <mergeCell ref="F27:M27"/>
-    <mergeCell ref="C35:E35"/>
-    <mergeCell ref="D36:M36"/>
-    <mergeCell ref="B37:M37"/>
+  <mergeCells count="15">
+    <mergeCell ref="B2:O2"/>
+    <mergeCell ref="B3:O3"/>
+    <mergeCell ref="B4:O4"/>
+    <mergeCell ref="E5:O5"/>
+    <mergeCell ref="B6:O6"/>
+    <mergeCell ref="H7:O7"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="E16:O16"/>
+    <mergeCell ref="B17:O17"/>
     <mergeCell ref="B7:B8"/>
-    <mergeCell ref="B27:B28"/>
     <mergeCell ref="C7:C8"/>
-    <mergeCell ref="C27:C28"/>
     <mergeCell ref="D7:D8"/>
-    <mergeCell ref="D27:D28"/>
     <mergeCell ref="E7:E8"/>
-    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F7:F8"/>
+    <mergeCell ref="G7:G8"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.393700787401575" right="0.393700787401575" top="0.590551181102362" bottom="0.590551181102362" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1818,9 +1598,8 @@
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6"/>
   <sheetData/>
-  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertRows="0" insertColumns="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511805555555556" footer="0.511805555555556"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" useFirstPageNumber="1" errors="NA" horizontalDpi="600"/>
   <headerFooter alignWithMargins="0"/>
@@ -1833,60 +1612,10 @@
     <pageSetUpPr autoPageBreaks="0"/>
   </sheetPr>
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="15.6"/>
   <sheetData/>
-  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertRows="0" insertColumns="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511805555555556" footer="0.511805555555556"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" useFirstPageNumber="1" errors="NA" horizontalDpi="600"/>
   <headerFooter alignWithMargins="0"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<woProps xmlns="https://web.wps.cn/et/2018/main" xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <woSheetsProps>
-    <woSheetProps sheetStid="1" interlineOnOff="0" interlineColor="0" isDbSheet="0" isDashBoardSheet="0" isDbDashBoardSheet="0" isFlexPaperSheet="0">
-      <cellprotection/>
-      <appEtDbRelations/>
-    </woSheetProps>
-    <woSheetProps sheetStid="2" interlineOnOff="0" interlineColor="0" isDbSheet="0" isDashBoardSheet="0" isDbDashBoardSheet="0" isFlexPaperSheet="0">
-      <cellprotection/>
-      <appEtDbRelations/>
-    </woSheetProps>
-    <woSheetProps sheetStid="3" interlineOnOff="0" interlineColor="0" isDbSheet="0" isDashBoardSheet="0" isDbDashBoardSheet="0" isFlexPaperSheet="0">
-      <cellprotection/>
-      <appEtDbRelations/>
-    </woSheetProps>
-  </woSheetsProps>
-  <woBookProps>
-    <bookSettings fileId="511666625487" isFilterShared="1" woEtMtcEnabled="0" coreConquerUserId="" isAutoUpdatePaused="0" filterType="conn" isMergeTasksAutoUpdate="0" isInserPicAsAttachment="0" supportDbFmlaDisp="0"/>
-  </woBookProps>
-</woProps>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<pixelators xmlns="https://web.wps.cn/et/2018/main" xmlns:s="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <pixelatorList sheetStid="1"/>
-  <pixelatorList sheetStid="2"/>
-  <pixelatorList sheetStid="3"/>
-  <pixelatorList sheetStid="4"/>
-</pixelators>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{06C82605-B75B-4693-9329-32AAD527C692}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="https://web.wps.cn/et/2018/main"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{224D003E-15C9-4FFE-AB16-9E66474EAE4E}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="https://web.wps.cn/et/2018/main"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>